<commit_message>
Train a Skill L1: fill standards/prescriptions from same-exercise template rows
Skill-sheet names with no exact template row now take the numbers of
the same exercise under its Upper Body template name (e.g. Full range
iron cross press = Iron Cross Press, DB Pull Hold = Cable Retraction twin).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015yWLLpzw9R1iGhMPWXgZsW
</commit_message>
<xml_diff>
--- a/Train_A_Skill/Level1_Train_A_Skill.xlsx
+++ b/Train_A_Skill/Level1_Train_A_Skill.xlsx
@@ -751,14 +751,14 @@
           <t>Full range iron cross press</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D13" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>10 reps at 5% of body weight</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>10 reps @ 2.5–5% BW</t>
         </is>
       </c>
     </row>
@@ -2532,14 +2532,14 @@
           <t>Full range iron cross press</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>10 reps at 5% of body weight</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>10 reps @ 2.5–5% BW</t>
         </is>
       </c>
     </row>
@@ -4509,14 +4509,14 @@
           <t>Full range iron cross press</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>10 reps at 5% of body weight</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>10 reps @ 2.5–5% BW</t>
         </is>
       </c>
     </row>
@@ -6396,14 +6396,14 @@
           <t>Full range iron cross press</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D12" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>10 reps at 5% of body weight</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>10 reps @ 2.5–5% BW</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Train a Skill L1: coach standards for the last open rows
Standards from Jesse (2026-10-26); prescriptions follow the matching
template pattern. No TBD rows left in Upper Body Strength.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015yWLLpzw9R1iGhMPWXgZsW
</commit_message>
<xml_diff>
--- a/Train_A_Skill/Level1_Train_A_Skill.xlsx
+++ b/Train_A_Skill/Level1_Train_A_Skill.xlsx
@@ -94,7 +94,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -118,11 +118,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFE599"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFEAF6E1"/>
       </patternFill>
     </fill>
@@ -139,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -168,22 +163,16 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -773,14 +762,14 @@
           <t>Rotational DB Push Hold</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D14" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>30% of bodyweight for 15 reps</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>10–15 reps @ 5–10% BW</t>
         </is>
       </c>
     </row>
@@ -898,14 +887,14 @@
           <t>2 Arm Retraction Rows</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>20 reps at horizontal angle</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>10–20 reps</t>
         </is>
       </c>
     </row>
@@ -1023,14 +1012,14 @@
           <t>Ring CARS</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D30" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>15 reps</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>5–15 reps</t>
         </is>
       </c>
     </row>
@@ -1979,14 +1968,14 @@
           <t>Weighted stick elbow rotations</t>
         </is>
       </c>
-      <c r="C92" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D92" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>5lb weighted bar for 10 reps</t>
+        </is>
+      </c>
+      <c r="D92" s="9" t="inlineStr">
+        <is>
+          <t>10 reps @ 2.5–5 lb</t>
         </is>
       </c>
     </row>
@@ -2001,14 +1990,14 @@
           <t>Banded Lat Pullover</t>
         </is>
       </c>
-      <c r="C93" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D93" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>20 reps medium resistance band</t>
+        </is>
+      </c>
+      <c r="D93" s="9" t="inlineStr">
+        <is>
+          <t>20 reps · light–medium resistance band</t>
         </is>
       </c>
     </row>
@@ -2554,14 +2543,14 @@
           <t>Rotational DB Push Hold</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>30% of bodyweight for 15 reps</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>10–15 reps @ 10–15% BW</t>
         </is>
       </c>
     </row>
@@ -2701,14 +2690,14 @@
           <t>2 Arm Retraction Rows</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D25" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>20 reps at horizontal angle</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>10–20 reps</t>
         </is>
       </c>
     </row>
@@ -2848,14 +2837,14 @@
           <t>Ring CARS</t>
         </is>
       </c>
-      <c r="C34" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D34" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>15 reps</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>5–15 reps</t>
         </is>
       </c>
     </row>
@@ -3936,14 +3925,14 @@
           <t>Weighted stick elbow rotations</t>
         </is>
       </c>
-      <c r="C102" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D102" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C102" s="8" t="inlineStr">
+        <is>
+          <t>5lb weighted bar for 10 reps</t>
+        </is>
+      </c>
+      <c r="D102" s="9" t="inlineStr">
+        <is>
+          <t>10 reps @ 2.5–5 lb</t>
         </is>
       </c>
     </row>
@@ -3958,14 +3947,14 @@
           <t>Banded Lat Pullover</t>
         </is>
       </c>
-      <c r="C103" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D103" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C103" s="8" t="inlineStr">
+        <is>
+          <t>20 reps medium resistance band</t>
+        </is>
+      </c>
+      <c r="D103" s="9" t="inlineStr">
+        <is>
+          <t>20 reps · light–medium resistance band</t>
         </is>
       </c>
     </row>
@@ -4531,14 +4520,14 @@
           <t>Rotational DB Push Hold</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>30% of bodyweight for 15 reps</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>10–15 reps @ 20–25% BW</t>
         </is>
       </c>
     </row>
@@ -4700,14 +4689,14 @@
           <t>2 Arm Retraction Rows</t>
         </is>
       </c>
-      <c r="C26" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>20 reps at horizontal angle</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>10–20 reps</t>
         </is>
       </c>
     </row>
@@ -4825,14 +4814,14 @@
           <t>Ring CARS</t>
         </is>
       </c>
-      <c r="C34" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D34" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>15 reps</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>5–15 reps</t>
         </is>
       </c>
     </row>
@@ -5891,14 +5880,14 @@
           <t>Weighted stick elbow rotations</t>
         </is>
       </c>
-      <c r="C101" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D101" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t>5lb weighted bar for 10 reps</t>
+        </is>
+      </c>
+      <c r="D101" s="9" t="inlineStr">
+        <is>
+          <t>10 reps @ 2.5–5 lb</t>
         </is>
       </c>
     </row>
@@ -5913,14 +5902,14 @@
           <t>Banded Lat Pullover</t>
         </is>
       </c>
-      <c r="C102" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D102" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C102" s="8" t="inlineStr">
+        <is>
+          <t>20 reps medium resistance band</t>
+        </is>
+      </c>
+      <c r="D102" s="9" t="inlineStr">
+        <is>
+          <t>20 reps · light–medium resistance band</t>
         </is>
       </c>
     </row>
@@ -6352,14 +6341,14 @@
           <t>Horizontal supinated support hold rings</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D10" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>45s hold fully horizontal scapula in protraction</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>20–45s</t>
         </is>
       </c>
     </row>
@@ -6418,14 +6407,14 @@
           <t>Rotational DB Push Hold</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D13" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>30% of bodyweight for 15 reps</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>10–15 reps @ 25–30% BW</t>
         </is>
       </c>
     </row>
@@ -7227,14 +7216,14 @@
           <t>Weighted stick elbow rotations</t>
         </is>
       </c>
-      <c r="C66" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D66" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>5lb weighted bar for 10 reps</t>
+        </is>
+      </c>
+      <c r="D66" s="9" t="inlineStr">
+        <is>
+          <t>10 reps @ 2.5–5 lb</t>
         </is>
       </c>
     </row>
@@ -7249,14 +7238,14 @@
           <t>Banded Lat Pullover</t>
         </is>
       </c>
-      <c r="C67" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D67" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>20 reps medium resistance band</t>
+        </is>
+      </c>
+      <c r="D67" s="9" t="inlineStr">
+        <is>
+          <t>20 reps · light–medium resistance band</t>
         </is>
       </c>
     </row>
@@ -7547,22 +7536,22 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>TEST: Contra-lateral Plank Hold</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>PASS: 30s hold each side</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>10–30s each side · 2 sets</t>
         </is>
@@ -7577,22 +7566,22 @@
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>TEST: Arching Hang Hold</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>PASS: 30s unbroken arching hang</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>10–30s · 2 sets</t>
         </is>
@@ -7607,22 +7596,22 @@
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>TEST: German Hang Hold Feet On Ground</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>PASS: 30s german hang (feet on ground)</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>10–30s · 2 sets</t>
         </is>
@@ -7637,22 +7626,22 @@
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>TEST: Chest to Wall Handstand Hold</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>PASS: 1 minute hold</t>
         </is>
       </c>
-      <c r="D15" s="15" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>20–60s · 2 sets  ✦</t>
         </is>
@@ -7667,22 +7656,22 @@
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>TEST: Tuck Support Hold- High bar</t>
         </is>
       </c>
-      <c r="C18" s="14" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
         <is>
           <t>PASS: 30 second hold</t>
         </is>
       </c>
-      <c r="D18" s="15" t="inlineStr">
+      <c r="D18" s="13" t="inlineStr">
         <is>
           <t>10–30s · 2 sets  ✦</t>
         </is>
@@ -7697,22 +7686,22 @@
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>TEST: Hanging L Sit</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>PASS: 30 second hold</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>10–30s · 2 sets  ✦</t>
         </is>
@@ -7727,44 +7716,44 @@
       </c>
     </row>
     <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>TEST: High Lizard Crawl-with push-up</t>
         </is>
       </c>
-      <c r="C24" s="14" t="inlineStr">
+      <c r="C24" s="12" t="inlineStr">
         <is>
           <t>PASS: 12 reps full range</t>
         </is>
       </c>
-      <c r="D24" s="15" t="inlineStr">
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>6–12 reps · 2 sets</t>
         </is>
       </c>
     </row>
     <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>TEST: Rotational High Lizard Crawl-with push-up</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>PASS: 12 reps full range</t>
         </is>
       </c>
-      <c r="D25" s="15" t="inlineStr">
+      <c r="D25" s="13" t="inlineStr">
         <is>
           <t>6–12 reps · 2 sets</t>
         </is>
@@ -7779,22 +7768,22 @@
       </c>
     </row>
     <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="12" t="inlineStr">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>TEST: Ring Pull: 2 Arm Feet Elevated</t>
         </is>
       </c>
-      <c r="C28" s="14" t="inlineStr">
+      <c r="C28" s="12" t="inlineStr">
         <is>
           <t>PASS: 10 reps feet elevated</t>
         </is>
       </c>
-      <c r="D28" s="15" t="inlineStr">
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>4–10 reps · 2 sets</t>
         </is>
@@ -7809,22 +7798,22 @@
       </c>
     </row>
     <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B31" s="13" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>TEST: Pike Elevated HSPU</t>
         </is>
       </c>
-      <c r="C31" s="14" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>PASS: 10 reps</t>
         </is>
       </c>
-      <c r="D31" s="15" t="inlineStr">
+      <c r="D31" s="13" t="inlineStr">
         <is>
           <t>4–10 reps · 2 sets  ✦</t>
         </is>
@@ -7839,22 +7828,22 @@
       </c>
     </row>
     <row r="34" ht="24" customHeight="1">
-      <c r="A34" s="12" t="inlineStr">
+      <c r="A34" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>TEST: Box/ Bar Push: 2 Arm Dip</t>
         </is>
       </c>
-      <c r="C34" s="14" t="inlineStr">
+      <c r="C34" s="12" t="inlineStr">
         <is>
           <t>PASS: 10 reps past 90°</t>
         </is>
       </c>
-      <c r="D34" s="15" t="inlineStr">
+      <c r="D34" s="13" t="inlineStr">
         <is>
           <t>4–10 reps past 90° · 2 sets  ✦</t>
         </is>
@@ -7869,44 +7858,44 @@
       </c>
     </row>
     <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="12" t="inlineStr">
+      <c r="A37" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>TEST: Ring/ Bar Chinup</t>
         </is>
       </c>
-      <c r="C37" s="14" t="inlineStr">
+      <c r="C37" s="12" t="inlineStr">
         <is>
           <t>PASS: 5 reps</t>
         </is>
       </c>
-      <c r="D37" s="15" t="inlineStr">
+      <c r="D37" s="13" t="inlineStr">
         <is>
           <t>1–5 reps · 2 sets  ✦</t>
         </is>
       </c>
     </row>
     <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="12" t="inlineStr">
+      <c r="A38" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
+      <c r="B38" s="11" t="inlineStr">
         <is>
           <t>TEST: Ring/ Bar Pullups</t>
         </is>
       </c>
-      <c r="C38" s="14" t="inlineStr">
+      <c r="C38" s="12" t="inlineStr">
         <is>
           <t>PASS: 5 reps</t>
         </is>
       </c>
-      <c r="D38" s="15" t="inlineStr">
+      <c r="D38" s="13" t="inlineStr">
         <is>
           <t>1–5 reps · 2 sets  ✦</t>
         </is>

</xml_diff>